<commit_message>
planilha de horas trabalhada
valter trabalhou
</commit_message>
<xml_diff>
--- a/tcc-documentacao/Planejamento/planilhas/horas-trabalhadas-tcc.xlsx
+++ b/tcc-documentacao/Planejamento/planilhas/horas-trabalhadas-tcc.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alunoinfo\Desktop\tcc\tcc-etec\tcc-documentacao\Planejamento\planilhas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alunoinfo\Desktop\Nova pasta\tcc-etec\tcc-documentacao\Planejamento\planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{415AA6D5-26C0-47CA-BB85-8052132C9BF4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A08EEFF7-CB37-4EF7-90D8-7DFB95CB635A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -645,19 +645,21 @@
       <c r="C5" s="4">
         <v>1</v>
       </c>
-      <c r="D5" s="4"/>
+      <c r="D5" s="4">
+        <v>1</v>
+      </c>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J5" s="5">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="2:12">
@@ -667,7 +669,9 @@
       <c r="C6" s="4">
         <v>0</v>
       </c>
-      <c r="D6" s="4"/>
+      <c r="D6" s="4">
+        <v>0</v>
+      </c>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4">

</xml_diff>

<commit_message>
mapa de api esboçado
</commit_message>
<xml_diff>
--- a/tcc-documentacao/Planejamento/planilhas/horas-trabalhadas-tcc.xlsx
+++ b/tcc-documentacao/Planejamento/planilhas/horas-trabalhadas-tcc.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alunoinfo\Desktop\tcc\tcc-etec\tcc-documentacao\Planejamento\planilhas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alunoinfo\Desktop\Nova pasta\tcc-etec\tcc-documentacao\Planejamento\planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80F2D41E-3AD3-4EDE-88B6-E696348C4483}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9535E9CB-4CF7-4582-8037-CD900A5B2D01}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -651,19 +651,19 @@
         <v>2</v>
       </c>
       <c r="E5" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5" s="4"/>
       <c r="G5" s="4">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J5" s="5">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="2:12">

</xml_diff>